<commit_message>
Added DDT Setup for Login
</commit_message>
<xml_diff>
--- a/TestData/Testdata.xlsx
+++ b/TestData/Testdata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="positive" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>Admin</t>
   </si>
@@ -29,6 +29,33 @@
   </si>
   <si>
     <t>admin123</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>failure</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>ExpectedResult</t>
+  </si>
+  <si>
+    <t>username_required</t>
+  </si>
+  <si>
+    <t>both_required</t>
+  </si>
+  <si>
+    <t>password_required</t>
   </si>
 </sst>
 </file>
@@ -346,15 +373,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>